<commit_message>
Generate Gerber NC Drill for ordering
</commit_message>
<xml_diff>
--- a/Project Outputs for Digital_Optical_Daughter_12Tx_1vXX/BOM/BOM_Digital_Optical_Daughter_12Tx_1vXX_1v01.xlsx
+++ b/Project Outputs for Digital_Optical_Daughter_12Tx_1vXX/BOM/BOM_Digital_Optical_Daughter_12Tx_1vXX_1v01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\Documents\Altium\UltraZOhm\Optical Daughter\Project Outputs for Digital_Optical_Daughter_12Tx_1vXX\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{84AF2AEA-BC0B-4EBB-8CBC-7024EA3BE460}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C492F198-A743-41E2-942E-6C26E0F7DA76}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11385" xr2:uid="{0BA43911-77FF-4DF0-AF38-CB4748271ACF}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="11385" xr2:uid="{25785278-4FD5-4C88-A4ED-3456E73B401C}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_Digital_Optical_Daughter_12" sheetId="1" r:id="rId1"/>
@@ -753,7 +753,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C5009F5-85F5-41AA-8352-363985DB2C7E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{604A1E43-E62E-4C00-BE7F-F0FF5F619B95}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>

</xml_diff>